<commit_message>
Extensive Dashboard annotations: Added help-text notes to Ledger, Weights, and Diagnostics for better self-documentation
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -166,6 +166,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Ross Wait</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Estimated Tax Payments Ledger: Record all tax payments made OUTSIDE of your W-2 withholding here. This is the source of truth for clearing shortfalls in the Action Center.</t>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>Calculated Estimate: The target amount recommended by the orchestrator based on pro-rated future projections.</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>Actual Payment Made: IMPORTANT: Enter the actual dollar amount sent to the IRS/FTB. This value is subtracted from your 'DUE NOW' totals.</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>Note: Use this to track voucher numbers, payment confirmation IDs, or intended quarters.</t>
+      </text>
+    </comment>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Safe Harbor (Fed): Enter your total tax from last year's Form 1040 (Line 24 minus Line 19).</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Safe Harbor (CA): Enter your total tax from last year's Form 540.</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Manual Offset: Adjust total income for one-off events (bonuses, sabbaticals) that aren't recurring in your snapshots.</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
+      <text>
+        <t>Weight: 1.0 = normal. &lt; 1.0 reduces projected future income. &gt; 1.0 increases it.</t>
+      </text>
+    </comment>
+    <comment ref="I15" authorId="0" shapeId="0">
+      <text>
+        <t>Diagnostics: A real-time verification of your tax health. Check effective rates to see your blended tax burden.</t>
+      </text>
+    </comment>
+    <comment ref="I18" authorId="0" shapeId="0">
+      <text>
+        <t>Effective Fed Rate: Total projected Federal Tax divided by Federal AGI. (Standardized against Fed AGI for comparability).</t>
+      </text>
+    </comment>
+    <comment ref="I19" authorId="0" shapeId="0">
+      <text>
+        <t>Effective CA Rate: Total projected California Tax divided by Federal AGI. (Standardized against Fed AGI for comparability).</t>
+      </text>
+    </comment>
+    <comment ref="I28" authorId="0" shapeId="0">
+      <text>
+        <t>HSA Audit: Ensures HSA contributions are effectively added back to California income (as they are not state-level deductions).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1602,6 +1672,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Final UX & Content refinement: Action Center styling, Ledger 'Required' labeling, and clean in-cell documentation
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -45,7 +45,7 @@
       <color rgb="00FF0000"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -60,12 +60,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -73,24 +79,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -176,62 +200,77 @@
   <commentList>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Estimated Tax Payments Ledger: Record all tax payments made OUTSIDE of your W-2 withholding here. This is the source of truth for clearing shortfalls in the Action Center.</t>
+        <t>Record your quarterly estimated tax payments made directly to the IRS or FTB here. This is the primary source of truth for tracking payments made outside of payroll withholding.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>The high-visibility focal point for immediate tax obligations. Values here update automatically based on today's date and your entered payments.</t>
       </text>
     </comment>
     <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>Calculated Estimate: The target amount recommended by the orchestrator based on pro-rated future projections.</t>
+        <t>An automated guide for this deadline based on your current year-to-date data. You can use this as a guide for your payment, or override it by entering your actual payment in the next column.</t>
       </text>
     </comment>
     <comment ref="F2" authorId="0" shapeId="0">
       <text>
-        <t>Actual Payment Made: IMPORTANT: Enter the actual dollar amount sent to the IRS/FTB. This value is subtracted from your 'DUE NOW' totals.</t>
+        <t>ENTER PAYMENTS HERE. This field is REQUIRED to accurately calculate your 'DUE NOW' totals in the Action Center. This ensures the system recognizes your progress and doesn't double-count required taxes.</t>
       </text>
     </comment>
     <comment ref="G2" authorId="0" shapeId="0">
       <text>
-        <t>Note: Use this to track voucher numbers, payment confirmation IDs, or intended quarters.</t>
+        <t>Track payment confirmation numbers, specific quarterly intent, or voucher details here.</t>
       </text>
     </comment>
     <comment ref="B4" authorId="0" shapeId="0">
       <text>
-        <t>Safe Harbor (Fed): Enter your total tax from last year's Form 1040 (Line 24 minus Line 19).</t>
+        <t>Enter your total tax from last year's Federal Form 1040 (typically Line 24 minus Line 19).</t>
       </text>
     </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Safe Harbor (CA): Enter your total tax from last year's Form 540.</t>
+        <t>Enter your total tax from last year's California Form 540.</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>Manual Offset: Adjust total income for one-off events (bonuses, sabbaticals) that aren't recurring in your snapshots.</t>
+        <t>Adjust total income for one-off events like bonuses or unpaid leave that aren't recurring in your payroll snapshots.</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
       <text>
-        <t>Weight: 1.0 = normal. &lt; 1.0 reduces projected future income. &gt; 1.0 increases it.</t>
+        <t>1.0 = normal earnings. Use &lt; 1.0 if you expect to stop working. Use &gt; 1.0 if you expect a year-end windfall.</t>
       </text>
     </comment>
     <comment ref="I15" authorId="0" shapeId="0">
       <text>
-        <t>Diagnostics: A real-time verification of your tax health. Check effective rates to see your blended tax burden.</t>
+        <t>A real-time health check on your tax situation. Verify your Effective Rates and Brackets to ensure the model matches your expectations.</t>
+      </text>
+    </comment>
+    <comment ref="I16" authorId="0" shapeId="0">
+      <text>
+        <t>Specifies if the system is currently targeting 110% of last year's tax (Safe Harbor) or 90% of your current forecast (Forecast), prioritizing the lower baseline for your safety.</t>
       </text>
     </comment>
     <comment ref="I18" authorId="0" shapeId="0">
       <text>
-        <t>Effective Fed Rate: Total projected Federal Tax divided by Federal AGI. (Standardized against Fed AGI for comparability).</t>
+        <t>Total projected Federal Tax divided by Federal AGI. (Standardized against Federal AGI for comparability).</t>
       </text>
     </comment>
     <comment ref="I19" authorId="0" shapeId="0">
       <text>
-        <t>Effective CA Rate: Total projected California Tax divided by Federal AGI. (Standardized against Fed AGI for comparability).</t>
+        <t>Total projected California Tax divided by Federal AGI. (Standardized against Federal AGI for comparability).</t>
+      </text>
+    </comment>
+    <comment ref="I21" authorId="0" shapeId="0">
+      <text>
+        <t>The highest tax rate applied to your last dollar of California income.</t>
       </text>
     </comment>
     <comment ref="I28" authorId="0" shapeId="0">
       <text>
-        <t>HSA Audit: Ensures HSA contributions are effectively added back to California income (as they are not state-level deductions).</t>
+        <t>Confirms that HSA contributions are successfully added back to California income (as they are not deductible at the state level).</t>
       </text>
     </comment>
   </commentList>
@@ -536,7 +575,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Universal Tax Orchestrator - Quick Start Guide</t>
+          <t>Quick Start Guide</t>
         </is>
       </c>
     </row>
@@ -560,7 +599,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Step 3: Enter your 'Prior Year Tax' liability in the Dashboard (Section 1) to enable Safe Harbor targets.</t>
+          <t>Step 3: Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
         </is>
       </c>
     </row>
@@ -575,9 +614,9 @@
       <c r="A7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>IMPORTANT NOTES &amp; SIMPLIFICATIONS:</t>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Important Notes</t>
         </is>
       </c>
     </row>
@@ -598,7 +637,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>3. Burn Rate Projections: The engine pro-rates your remaining annual income based on the days elapsed between Jan 1 and your latest snapshot date.</t>
+          <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
         </is>
       </c>
     </row>
@@ -627,8 +666,8 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
@@ -646,11 +685,12 @@
           <t>Estimated Tax Payments Ledger</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>PAYMENT ACTION CENTER</t>
         </is>
       </c>
+      <c r="J1" s="4" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -658,7 +698,7 @@
           <t>Filing Status (Single)</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -670,12 +710,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Calculated Estimate</t>
+          <t>Calculated Estimate (Optional)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Actual Payment Made</t>
+          <t>Actual Payment Made (Required)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -683,12 +723,12 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>FED DUE NOW:</t>
         </is>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="7">
         <f>IFS(B9&lt;=DATE(B8,4,15), C55, B9&lt;=DATE(B8,6,15), C56, B9&lt;=DATE(B8,9,15), C57, TRUE, C58)</f>
         <v/>
       </c>
@@ -699,27 +739,27 @@
           <t>Dependents (Under 17)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>04/15/2026</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>Fed Q1</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>BY DEADLINE:</t>
         </is>
       </c>
-      <c r="J3">
+      <c r="J3" s="4">
         <f>IFS(B9&lt;=DATE(B8,4,15), "04/15/"&amp;B8, B9&lt;=DATE(B8,6,15), "06/15/"&amp;B8, B9&lt;=DATE(B8,9,15), "09/15/"&amp;B8, TRUE, "01/15/"&amp;(B8+1))</f>
         <v/>
       </c>
@@ -730,27 +770,27 @@
           <t>Prior Year Fed Tax (Safe Harbor)</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>04/15/2026</t>
         </is>
       </c>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>CA Q1</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Next FED Target:</t>
         </is>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="13">
         <f>IFS(B9&lt;=DATE(B8,4,15), B55, B9&lt;=DATE(B8,6,15), B56, B9&lt;=DATE(B8,9,15), B57, TRUE, B58)</f>
         <v/>
       </c>
@@ -761,27 +801,27 @@
           <t>Prior Year CA Tax (Safe Harbor)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>06/15/2026</t>
         </is>
       </c>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Fed Q2</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>FED Payments YTD:</t>
         </is>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="13">
         <f>B50</f>
         <v/>
       </c>
@@ -792,27 +832,27 @@
           <t>Estimated Fed Itemized Deduction</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>06/15/2026</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>CA Q2</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>FED Status:</t>
         </is>
       </c>
-      <c r="J6">
+      <c r="J6" s="4">
         <f>IF(J5&gt;=J4, "✅ Met (Surplus: " &amp; TEXT(J5-J4, "$#,##0") &amp; ")", "🔴 Shortfall (" &amp; TEXT(J4-J5, "$#,##0") &amp; ")")</f>
         <v/>
       </c>
@@ -823,22 +863,23 @@
           <t>Estimated CA Itemized Deduction</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>09/15/2026</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Fed Q3</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -846,27 +887,27 @@
           <t>Tax Year</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>2026</v>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>09/15/2026</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>CA Q3</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>CA DUE NOW:</t>
         </is>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="7">
         <f>IFS(B9&lt;=DATE(B8,4,15), C61, B9&lt;=DATE(B8,6,15), C62, B9&lt;=DATE(B8,9,15), C63, TRUE, C64)</f>
         <v/>
       </c>
@@ -877,52 +918,52 @@
           <t>Status Date</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="14">
         <f>TODAY()</f>
         <v/>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>01/15/2027</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>Fed Q4</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>BY DEADLINE:</t>
         </is>
       </c>
-      <c r="J9">
+      <c r="J9" s="4">
         <f>IFS(B9&lt;=DATE(B8,4,15), "04/15/"&amp;B8, B9&lt;=DATE(B8,6,15), "06/15/"&amp;B8, B9&lt;=DATE(B8,9,15), "09/15/"&amp;B8, TRUE, "01/15/"&amp;(B8+1))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>01/15/2027</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>CA Q4</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Next CA Target:</t>
         </is>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="13">
         <f>IFS(B9&lt;=DATE(B8,4,15), B61, B9&lt;=DATE(B8,6,15), B62, B9&lt;=DATE(B8,9,15), B63, TRUE, B64)</f>
         <v/>
       </c>
@@ -934,12 +975,12 @@
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>CA Payments YTD:</t>
         </is>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="13">
         <f>B52</f>
         <v/>
       </c>
@@ -950,16 +991,16 @@
           <t>Manual Income Offset ($)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>CA Status:</t>
         </is>
       </c>
-      <c r="J12">
+      <c r="J12" s="4">
         <f>IF(J11&gt;=J10, "✅ Met (Surplus: " &amp; TEXT(J11-J10, "$#,##0") &amp; ")", "🔴 Shortfall (" &amp; TEXT(J10-J11, "$#,##0") &amp; ")")</f>
         <v/>
       </c>
@@ -970,11 +1011,12 @@
           <t>Future Income Weight (%)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="15" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -982,7 +1024,7 @@
           <t>Remaining Year Wage Income</t>
         </is>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="12">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
@@ -995,7 +1037,7 @@
           <t>Remaining Year Deductions</t>
         </is>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="12">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
@@ -1042,7 +1084,7 @@
           <t>Total Projected Wage Income</t>
         </is>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="16">
         <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
@@ -1052,7 +1094,7 @@
           <t>Effective Fed Rate:</t>
         </is>
       </c>
-      <c r="J18" s="13">
+      <c r="J18" s="17">
         <f>B46 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1063,7 +1105,7 @@
           <t>Federal W-2 State Wages</t>
         </is>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="16">
         <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
@@ -1073,7 +1115,7 @@
           <t>Effective CA Rate:</t>
         </is>
       </c>
-      <c r="J19" s="13">
+      <c r="J19" s="17">
         <f>B37 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1084,7 +1126,7 @@
           <t>CA W-2 State Wages</t>
         </is>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="16">
         <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
@@ -1094,7 +1136,7 @@
           <t>Marginal Fed Bracket:</t>
         </is>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="17">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1105,7 +1147,7 @@
           <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="16">
         <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
@@ -1115,7 +1157,7 @@
           <t>Marginal CA Bracket:</t>
         </is>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="17">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1126,7 +1168,7 @@
           <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="16">
         <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
@@ -1147,7 +1189,7 @@
           <t>Total Projected Federal AGI</t>
         </is>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="16">
         <f>B19 + B21 + B22</f>
         <v/>
       </c>
@@ -1160,7 +1202,7 @@
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="16">
         <f>B20 + B21 + B22</f>
         <v/>
       </c>
@@ -1189,7 +1231,7 @@
         </is>
       </c>
       <c r="J26">
-        <f>IF(OR(MAX('Wage Snapshots'!A:A)=0, (B9 - MAX('Wage Snapshots'!A:A)) &gt; 30), "!!! 30+ DAYS OLD !!!", "OK")</f>
+        <f>IF(OR(MAX('Wage Snapshots'!A:A)=0, (B9 - MAX('Wage Snapshots'!A:A)) &gt; 30), "🔴 !!! 30+ DAYS OLD !!!", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1199,7 +1241,7 @@
           <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
-      <c r="B27" s="10">
+      <c r="B27" s="16">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A3:A30, 'Tax Constants'!E3:E30, 0), B6)</f>
         <v/>
       </c>
@@ -1210,7 +1252,7 @@
         </is>
       </c>
       <c r="J27">
-        <f>IF(B4=0, "WARNING: FED MISSING", "OK")</f>
+        <f>IF(B4=0, "🔴 WARNING: FED MISSING", "OK")</f>
         <v/>
       </c>
     </row>
@@ -1220,7 +1262,7 @@
           <t>Ordinary Taxable Income</t>
         </is>
       </c>
-      <c r="B28" s="10">
+      <c r="B28" s="16">
         <f>MAX(0, B23 - B27 - B22)</f>
         <v/>
       </c>
@@ -1241,7 +1283,7 @@
           <t>Ordinary Income Tax</t>
         </is>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="16">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!A3:A30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1254,7 +1296,7 @@
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B30" s="10">
+      <c r="B30" s="16">
         <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!B34:B45, 'Tax Constants'!A34:A45=B2), FILTER('Tax Constants'!C34:C45, 'Tax Constants'!A34:A45=B2), 0, -1), 0)</f>
         <v/>
       </c>
@@ -1281,7 +1323,7 @@
           <t>CA Deduction Applied</t>
         </is>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="16">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A49:A84, 'Tax Constants'!E49:E84, 0), B7)</f>
         <v/>
       </c>
@@ -1294,7 +1336,7 @@
           <t>CA Taxable Income</t>
         </is>
       </c>
-      <c r="B34" s="10">
+      <c r="B34" s="16">
         <f>MAX(0, B24 - B33)</f>
         <v/>
       </c>
@@ -1307,7 +1349,7 @@
           <t>CA Regular Tax</t>
         </is>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="16">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!A49:A84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1320,7 +1362,7 @@
           <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
-      <c r="B36" s="10">
+      <c r="B36" s="16">
         <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
@@ -1333,7 +1375,7 @@
           <t>Total CA Liability</t>
         </is>
       </c>
-      <c r="B37" s="10">
+      <c r="B37" s="16">
         <f>B35 + B36</f>
         <v/>
       </c>
@@ -1360,7 +1402,7 @@
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="B40" s="10">
+      <c r="B40" s="16">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!B88:B91, 200000)</f>
         <v/>
       </c>
@@ -1373,7 +1415,7 @@
           <t>NIIT (Fed)</t>
         </is>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="16">
         <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
         <v/>
       </c>
@@ -1386,7 +1428,7 @@
           <t>Addl Medicare Threshold</t>
         </is>
       </c>
-      <c r="B42" s="10">
+      <c r="B42" s="16">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
@@ -1399,7 +1441,7 @@
           <t>Addl Medicare (Fed)</t>
         </is>
       </c>
-      <c r="B43" s="10">
+      <c r="B43" s="16">
         <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
         <v/>
       </c>
@@ -1412,7 +1454,7 @@
           <t>CTC Phaseout Start</t>
         </is>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="16">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
@@ -1425,7 +1467,7 @@
           <t>Child Tax Credit</t>
         </is>
       </c>
-      <c r="B45" s="10">
+      <c r="B45" s="16">
         <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
         <v/>
       </c>
@@ -1438,7 +1480,7 @@
           <t>Total Federal Liability</t>
         </is>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="16">
         <f>B29 + B30 + B41 + B43 - B45</f>
         <v/>
       </c>
@@ -1465,7 +1507,7 @@
           <t>Fed Target</t>
         </is>
       </c>
-      <c r="B49" s="10">
+      <c r="B49" s="16">
         <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
@@ -1478,7 +1520,7 @@
           <t>Total Fed Payments YTD</t>
         </is>
       </c>
-      <c r="B50" s="10">
+      <c r="B50" s="16">
         <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
@@ -1491,7 +1533,7 @@
           <t>CA Target</t>
         </is>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="16">
         <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
@@ -1504,7 +1546,7 @@
           <t>Total CA Payments YTD</t>
         </is>
       </c>
-      <c r="B52" s="10">
+      <c r="B52" s="16">
         <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
@@ -1518,7 +1560,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
-      <c r="C54" s="10" t="n"/>
+      <c r="C54" s="16" t="n"/>
       <c r="D54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
     </row>
@@ -1532,7 +1574,7 @@
         <f>B49 * 0.25</f>
         <v/>
       </c>
-      <c r="C55" s="10">
+      <c r="C55" s="16">
         <f>MAX(0, B55 - B50)</f>
         <v/>
       </c>
@@ -1549,7 +1591,7 @@
         <f>B49 * 0.5</f>
         <v/>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="16">
         <f>MAX(0, B56 - B50)</f>
         <v/>
       </c>
@@ -1566,7 +1608,7 @@
         <f>B49 * 0.75</f>
         <v/>
       </c>
-      <c r="C57" s="10">
+      <c r="C57" s="16">
         <f>MAX(0, B57 - B50)</f>
         <v/>
       </c>
@@ -1583,7 +1625,7 @@
         <f>B49 * 1.0</f>
         <v/>
       </c>
-      <c r="C58" s="10">
+      <c r="C58" s="16">
         <f>MAX(0, B58 - B50)</f>
         <v/>
       </c>
@@ -1592,13 +1634,13 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
-      <c r="C59" s="10" t="n"/>
+      <c r="C59" s="16" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
-      <c r="C60" s="10" t="n"/>
+      <c r="C60" s="16" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
@@ -1612,7 +1654,7 @@
         <f>B51 * 0.3</f>
         <v/>
       </c>
-      <c r="C61" s="10">
+      <c r="C61" s="16">
         <f>MAX(0, B61 - B52)</f>
         <v/>
       </c>
@@ -1629,7 +1671,7 @@
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C62" s="10">
+      <c r="C62" s="16">
         <f>MAX(0, B62 - B52)</f>
         <v/>
       </c>
@@ -1646,7 +1688,7 @@
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C63" s="10">
+      <c r="C63" s="16">
         <f>MAX(0, B63 - B52)</f>
         <v/>
       </c>
@@ -1663,7 +1705,7 @@
         <f>B51 * 1.0</f>
         <v/>
       </c>
-      <c r="C64" s="10">
+      <c r="C64" s="16">
         <f>MAX(0, B64 - B52)</f>
         <v/>
       </c>
@@ -1804,7 +1846,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table A: Federal Brackets (Ordinary Income - 2026)</t>
+          <t>Table A: Federal Brackets (Ordinary Income)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -2379,7 +2421,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Table B: Federal Capital Gains Brackets (2026)</t>
+          <t>Table B: Federal Capital Gains Brackets</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
@@ -2577,7 +2619,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Table C: California FTB Brackets (2026)</t>
+          <t>Table C: California FTB Brackets</t>
         </is>
       </c>
       <c r="D47" s="2" t="n"/>

</xml_diff>

<commit_message>
Refined Action Center UI: Removed borders and restored dark blue header styling
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -60,18 +60,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
         <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -79,41 +79,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -210,7 +195,7 @@
     </comment>
     <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>MANUAL ENTRY. This field is NOT auto-populated. It is provided as a convenience for you to manually log what the system recommended at the time of your payment for your records.</t>
+        <t>MANUAL ENTRY. This field is not auto-populated. It is provided as a convenience for you to manually log what the system recommended at the time of your payment for your records.</t>
       </text>
     </comment>
     <comment ref="F2" authorId="0" shapeId="0">
@@ -685,12 +670,12 @@
           <t>Estimated Tax Payments Ledger</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>PAYMENT ACTION CENTER</t>
         </is>
       </c>
-      <c r="J1" s="4" t="n"/>
+      <c r="J1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -698,7 +683,7 @@
           <t>Filing Status (Single)</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -723,12 +708,12 @@
           <t>Note</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>FED DUE NOW:</t>
         </is>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="5">
         <f>IFS(B9&lt;=DATE(B8,4,15), C55, B9&lt;=DATE(B8,6,15), C56, B9&lt;=DATE(B8,9,15), C57, TRUE, C58)</f>
         <v/>
       </c>
@@ -739,27 +724,27 @@
           <t>Dependents (Under 17)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>04/15/2026</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Fed Q1</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>BY DEADLINE:</t>
         </is>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="10">
         <f>IFS(B9&lt;=DATE(B8,4,15), "04/15/"&amp;B8, B9&lt;=DATE(B8,6,15), "06/15/"&amp;B8, B9&lt;=DATE(B8,9,15), "09/15/"&amp;B8, TRUE, "01/15/"&amp;(B8+1))</f>
         <v/>
       </c>
@@ -770,27 +755,27 @@
           <t>Prior Year Fed Tax (Safe Harbor)</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>04/15/2026</t>
         </is>
       </c>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>CA Q1</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Next FED Target:</t>
         </is>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="12">
         <f>IFS(B9&lt;=DATE(B8,4,15), B55, B9&lt;=DATE(B8,6,15), B56, B9&lt;=DATE(B8,9,15), B57, TRUE, B58)</f>
         <v/>
       </c>
@@ -801,27 +786,27 @@
           <t>Prior Year CA Tax (Safe Harbor)</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>06/15/2026</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Fed Q2</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>FED Payments YTD:</t>
         </is>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="12">
         <f>B50</f>
         <v/>
       </c>
@@ -832,27 +817,27 @@
           <t>Estimated Fed Itemized Deduction</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>06/15/2026</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>CA Q2</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>FED Status:</t>
         </is>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="10">
         <f>IF(J5&gt;=J4, "✅ Met (Surplus: " &amp; TEXT(J5-J4, "$#,##0") &amp; ")", "🔴 Shortfall (" &amp; TEXT(J4-J5, "$#,##0") &amp; ")")</f>
         <v/>
       </c>
@@ -863,23 +848,23 @@
           <t>Estimated CA Itemized Deduction</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>09/15/2026</t>
         </is>
       </c>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Fed Q3</t>
         </is>
       </c>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -887,27 +872,27 @@
           <t>Tax Year</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="3" t="n">
         <v>2026</v>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>09/15/2026</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>CA Q3</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>CA DUE NOW:</t>
         </is>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="5">
         <f>IFS(B9&lt;=DATE(B8,4,15), C61, B9&lt;=DATE(B8,6,15), C62, B9&lt;=DATE(B8,9,15), C63, TRUE, C64)</f>
         <v/>
       </c>
@@ -918,52 +903,52 @@
           <t>Status Date</t>
         </is>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="13">
         <f>TODAY()</f>
         <v/>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>01/15/2027</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Fed Q4</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>BY DEADLINE:</t>
         </is>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="10">
         <f>IFS(B9&lt;=DATE(B8,4,15), "04/15/"&amp;B8, B9&lt;=DATE(B8,6,15), "06/15/"&amp;B8, B9&lt;=DATE(B8,9,15), "09/15/"&amp;B8, TRUE, "01/15/"&amp;(B8+1))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>01/15/2027</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>CA Q4</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>Next CA Target:</t>
         </is>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="12">
         <f>IFS(B9&lt;=DATE(B8,4,15), B61, B9&lt;=DATE(B8,6,15), B62, B9&lt;=DATE(B8,9,15), B63, TRUE, B64)</f>
         <v/>
       </c>
@@ -975,12 +960,12 @@
         </is>
       </c>
       <c r="D11" s="2" t="n"/>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>CA Payments YTD:</t>
         </is>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="12">
         <f>B52</f>
         <v/>
       </c>
@@ -991,16 +976,16 @@
           <t>Manual Income Offset ($)</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n"/>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>CA Status:</t>
         </is>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="10">
         <f>IF(J11&gt;=J10, "✅ Met (Surplus: " &amp; TEXT(J11-J10, "$#,##0") &amp; ")", "🔴 Shortfall (" &amp; TEXT(J10-J11, "$#,##0") &amp; ")")</f>
         <v/>
       </c>
@@ -1011,12 +996,12 @@
           <t>Future Income Weight (%)</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="4" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1024,7 +1009,7 @@
           <t>Remaining Year Wage Income</t>
         </is>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!B:B) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
@@ -1037,7 +1022,7 @@
           <t>Remaining Year Deductions</t>
         </is>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="11">
         <f>IF(MAX('Wage Snapshots'!A:A)=0, 0, (SUM('Wage Snapshots'!C:D) / MAX(1, MAX('Wage Snapshots'!A:A) - DATE(B8,1,1))) * (DATE(B8,12,31) - MAX('Wage Snapshots'!A:A)))</f>
         <v/>
       </c>
@@ -1084,7 +1069,7 @@
           <t>Total Projected Wage Income</t>
         </is>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="15">
         <f>SUM('Wage Snapshots'!B:B) + (B14 * B13) + B12</f>
         <v/>
       </c>
@@ -1094,7 +1079,7 @@
           <t>Effective Fed Rate:</t>
         </is>
       </c>
-      <c r="J18" s="17">
+      <c r="J18" s="16">
         <f>B46 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1105,7 +1090,7 @@
           <t>Federal W-2 State Wages</t>
         </is>
       </c>
-      <c r="B19" s="16">
+      <c r="B19" s="15">
         <f>B18 - SUM('Wage Snapshots'!C:D) - (B15 * B13)</f>
         <v/>
       </c>
@@ -1115,7 +1100,7 @@
           <t>Effective CA Rate:</t>
         </is>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="16">
         <f>B37 / MAX(1, B23)</f>
         <v/>
       </c>
@@ -1126,7 +1111,7 @@
           <t>CA W-2 State Wages</t>
         </is>
       </c>
-      <c r="B20" s="16">
+      <c r="B20" s="15">
         <f>B18 - SUM('Wage Snapshots'!C:C) - (SUM('Wage Snapshots'!C:C)/MAX(1, SUM('Wage Snapshots'!C:D))) * B15 * B13</f>
         <v/>
       </c>
@@ -1136,7 +1121,7 @@
           <t>Marginal Fed Bracket:</t>
         </is>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="16">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1147,7 +1132,7 @@
           <t>Investment Ordinary (Div/Int + STG)</t>
         </is>
       </c>
-      <c r="B21" s="16">
+      <c r="B21" s="15">
         <f>SUM('Investment Income Snapshots'!C:C) + SUM('Investment Income Snapshots'!D:D)</f>
         <v/>
       </c>
@@ -1157,7 +1142,7 @@
           <t>Marginal CA Bracket:</t>
         </is>
       </c>
-      <c r="J21" s="17">
+      <c r="J21" s="16">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1168,7 +1153,7 @@
           <t>Investment Preferential (LTG Only)</t>
         </is>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="15">
         <f>SUM('Investment Income Snapshots'!E:E)</f>
         <v/>
       </c>
@@ -1189,7 +1174,7 @@
           <t>Total Projected Federal AGI</t>
         </is>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <f>B19 + B21 + B22</f>
         <v/>
       </c>
@@ -1202,7 +1187,7 @@
           <t>Total Projected CA AGI</t>
         </is>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="15">
         <f>B20 + B21 + B22</f>
         <v/>
       </c>
@@ -1241,7 +1226,7 @@
           <t>Deduction Applied (Max Std/Item)</t>
         </is>
       </c>
-      <c r="B27" s="16">
+      <c r="B27" s="15">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A3:A30, 'Tax Constants'!E3:E30, 0), B6)</f>
         <v/>
       </c>
@@ -1262,7 +1247,7 @@
           <t>Ordinary Taxable Income</t>
         </is>
       </c>
-      <c r="B28" s="16">
+      <c r="B28" s="15">
         <f>MAX(0, B23 - B27 - B22)</f>
         <v/>
       </c>
@@ -1283,7 +1268,7 @@
           <t>Ordinary Income Tax</t>
         </is>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="15">
         <f>XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!C3:C30, 'Tax Constants'!A3:A30=B2), 0, -1) + (B28 - XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), 0, -1)) * XLOOKUP(B28, FILTER('Tax Constants'!B3:B30, 'Tax Constants'!A3:A30=B2), FILTER('Tax Constants'!D3:D30, 'Tax Constants'!A3:A30=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1296,7 +1281,7 @@
           <t>Capital Gains Tax</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <f>IF(B22&gt;0, B22 * XLOOKUP(B28+B22, FILTER('Tax Constants'!B34:B45, 'Tax Constants'!A34:A45=B2), FILTER('Tax Constants'!C34:C45, 'Tax Constants'!A34:A45=B2), 0, -1), 0)</f>
         <v/>
       </c>
@@ -1323,7 +1308,7 @@
           <t>CA Deduction Applied</t>
         </is>
       </c>
-      <c r="B33" s="16">
+      <c r="B33" s="15">
         <f>MAX(XLOOKUP(B2, 'Tax Constants'!A49:A84, 'Tax Constants'!E49:E84, 0), B7)</f>
         <v/>
       </c>
@@ -1336,7 +1321,7 @@
           <t>CA Taxable Income</t>
         </is>
       </c>
-      <c r="B34" s="16">
+      <c r="B34" s="15">
         <f>MAX(0, B24 - B33)</f>
         <v/>
       </c>
@@ -1349,7 +1334,7 @@
           <t>CA Regular Tax</t>
         </is>
       </c>
-      <c r="B35" s="16">
+      <c r="B35" s="15">
         <f>XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!C49:C84, 'Tax Constants'!A49:A84=B2), 0, -1) + (B34 - XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), 0, -1)) * XLOOKUP(B34, FILTER('Tax Constants'!B49:B84, 'Tax Constants'!A49:A84=B2), FILTER('Tax Constants'!D49:D84, 'Tax Constants'!A49:A84=B2), 0, -1)</f>
         <v/>
       </c>
@@ -1362,7 +1347,7 @@
           <t>CA MH Surcharge (1%)</t>
         </is>
       </c>
-      <c r="B36" s="16">
+      <c r="B36" s="15">
         <f>IF(B34 &gt; 1000000, (B34 - 1000000) * 0.01, 0)</f>
         <v/>
       </c>
@@ -1375,7 +1360,7 @@
           <t>Total CA Liability</t>
         </is>
       </c>
-      <c r="B37" s="16">
+      <c r="B37" s="15">
         <f>B35 + B36</f>
         <v/>
       </c>
@@ -1402,7 +1387,7 @@
           <t>NIIT Threshold</t>
         </is>
       </c>
-      <c r="B40" s="16">
+      <c r="B40" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!B88:B91, 200000)</f>
         <v/>
       </c>
@@ -1415,7 +1400,7 @@
           <t>NIIT (Fed)</t>
         </is>
       </c>
-      <c r="B41" s="16">
+      <c r="B41" s="15">
         <f>IF(B23 &gt; B40, 0.038 * MIN(B23-B40, B21+B22), 0)</f>
         <v/>
       </c>
@@ -1428,7 +1413,7 @@
           <t>Addl Medicare Threshold</t>
         </is>
       </c>
-      <c r="B42" s="16">
+      <c r="B42" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!C88:C91, 200000)</f>
         <v/>
       </c>
@@ -1441,7 +1426,7 @@
           <t>Addl Medicare (Fed)</t>
         </is>
       </c>
-      <c r="B43" s="16">
+      <c r="B43" s="15">
         <f>IF(B18 &gt; B42, 0.009 * (B18-B42), 0)</f>
         <v/>
       </c>
@@ -1454,7 +1439,7 @@
           <t>CTC Phaseout Start</t>
         </is>
       </c>
-      <c r="B44" s="16">
+      <c r="B44" s="15">
         <f>XLOOKUP(B2, 'Tax Constants'!A88:A91, 'Tax Constants'!D88:D91, 200000)</f>
         <v/>
       </c>
@@ -1467,7 +1452,7 @@
           <t>Child Tax Credit</t>
         </is>
       </c>
-      <c r="B45" s="16">
+      <c r="B45" s="15">
         <f>IF(B23 &gt; B44, MAX(0, (B3*2000)-((B23-B44)/1000)*50), B3*2000)</f>
         <v/>
       </c>
@@ -1480,7 +1465,7 @@
           <t>Total Federal Liability</t>
         </is>
       </c>
-      <c r="B46" s="16">
+      <c r="B46" s="15">
         <f>B29 + B30 + B41 + B43 - B45</f>
         <v/>
       </c>
@@ -1507,7 +1492,7 @@
           <t>Fed Target</t>
         </is>
       </c>
-      <c r="B49" s="16">
+      <c r="B49" s="15">
         <f>IF(B4=0, B46 * 0.9, MIN(B46 * 0.9, B4 * 1.1))</f>
         <v/>
       </c>
@@ -1520,7 +1505,7 @@
           <t>Total Fed Payments YTD</t>
         </is>
       </c>
-      <c r="B50" s="16">
+      <c r="B50" s="15">
         <f>SUM('Wage Snapshots'!E:E) + SUMIFS(F3:F10, G3:G10, "Fed*")</f>
         <v/>
       </c>
@@ -1533,7 +1518,7 @@
           <t>CA Target</t>
         </is>
       </c>
-      <c r="B51" s="16">
+      <c r="B51" s="15">
         <f>IF(B5=0, B37 * 0.8, MIN(B37 * 0.8, B5 * 1.1))</f>
         <v/>
       </c>
@@ -1546,7 +1531,7 @@
           <t>Total CA Payments YTD</t>
         </is>
       </c>
-      <c r="B52" s="16">
+      <c r="B52" s="15">
         <f>SUM('Wage Snapshots'!F:F) + SUMIFS(F3:F10, G3:G10, "CA*")</f>
         <v/>
       </c>
@@ -1560,7 +1545,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
-      <c r="C54" s="16" t="n"/>
+      <c r="C54" s="15" t="n"/>
       <c r="D54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
     </row>
@@ -1574,7 +1559,7 @@
         <f>B49 * 0.25</f>
         <v/>
       </c>
-      <c r="C55" s="16">
+      <c r="C55" s="15">
         <f>MAX(0, B55 - B50)</f>
         <v/>
       </c>
@@ -1591,7 +1576,7 @@
         <f>B49 * 0.5</f>
         <v/>
       </c>
-      <c r="C56" s="16">
+      <c r="C56" s="15">
         <f>MAX(0, B56 - B50)</f>
         <v/>
       </c>
@@ -1608,7 +1593,7 @@
         <f>B49 * 0.75</f>
         <v/>
       </c>
-      <c r="C57" s="16">
+      <c r="C57" s="15">
         <f>MAX(0, B57 - B50)</f>
         <v/>
       </c>
@@ -1625,7 +1610,7 @@
         <f>B49 * 1.0</f>
         <v/>
       </c>
-      <c r="C58" s="16">
+      <c r="C58" s="15">
         <f>MAX(0, B58 - B50)</f>
         <v/>
       </c>
@@ -1634,13 +1619,13 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
-      <c r="C59" s="16" t="n"/>
+      <c r="C59" s="15" t="n"/>
       <c r="D59" s="2" t="n"/>
       <c r="I59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
-      <c r="C60" s="16" t="n"/>
+      <c r="C60" s="15" t="n"/>
       <c r="D60" s="2" t="n"/>
       <c r="I60" s="2" t="n"/>
     </row>
@@ -1654,7 +1639,7 @@
         <f>B51 * 0.3</f>
         <v/>
       </c>
-      <c r="C61" s="16">
+      <c r="C61" s="15">
         <f>MAX(0, B61 - B52)</f>
         <v/>
       </c>
@@ -1671,7 +1656,7 @@
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C62" s="16">
+      <c r="C62" s="15">
         <f>MAX(0, B62 - B52)</f>
         <v/>
       </c>
@@ -1688,7 +1673,7 @@
         <f>B51 * 0.7</f>
         <v/>
       </c>
-      <c r="C63" s="16">
+      <c r="C63" s="15">
         <f>MAX(0, B63 - B52)</f>
         <v/>
       </c>
@@ -1705,7 +1690,7 @@
         <f>B51 * 1.0</f>
         <v/>
       </c>
-      <c r="C64" s="16">
+      <c r="C64" s="15">
         <f>MAX(0, B64 - B52)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Added comments for Stale Snapshots and Prior Year Data warnings
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -251,6 +251,16 @@
     <comment ref="I21" authorId="0" shapeId="0">
       <text>
         <t>The highest tax rate applied to your last dollar of California income.</t>
+      </text>
+    </comment>
+    <comment ref="I26" authorId="0" shapeId="0">
+      <text>
+        <t>Alerts you if your latest snapshot is more than 30 days old. Keeping this current ensures accurately pro-rated future predictions.</t>
+      </text>
+    </comment>
+    <comment ref="I27" authorId="0" shapeId="0">
+      <text>
+        <t>Critical for Safe Harbor targeting. Warns you if your prior-year tax liability is missing from the Configuration section (B4/B5).</t>
       </text>
     </comment>
     <comment ref="I28" authorId="0" shapeId="0">

</xml_diff>

<commit_message>
Fixed Instructions tab styling: Restricted section headers to specific rows and prevented random keyword matches
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -575,69 +575,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Step 1: Enter your latest YTD paystub details in the 'Wage Snapshots' tab.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Step 2: Enter your latest YTD brokerage totals in 'Investment Income Snapshots'.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Step 3: Enter your 'Prior Year Tax' liability in the Dashboard to enable Safe Harbor targets.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Step 4: Check the 'PAYMENT ACTION CENTER' on the Dashboard for immediate payment requirements.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Important Notes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>1. Investment Income: All dividends and interest are combined and taxed as Ordinary Income for a safe, conservative projection.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2. HSA (California): HSA contributions are automatically added back to CA state income as they are not deductible in California.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>3. Income Projections: The engine pro-rates your remaining annual income based on the days elapsed since Jan 1. You can adjust these projections by entering values into 'Manual Income Offset' or 'Future Income Weight' in Section 1.5 of the Dashboard.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>4. YTD Methodology: Always use Year-to-Date (YTD) totals from your statements. Overwrite existing rows as new statements arrive.</t>
         </is>
@@ -1851,7 +1851,7 @@
       <c r="F1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1866,7 +1866,7 @@
           <t>Base Tax</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Marginal Rate</t>
         </is>
@@ -1878,7 +1878,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1889,7 +1889,7 @@
       <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>0.1</v>
       </c>
       <c r="E3" t="n">
@@ -1897,7 +1897,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1908,7 +1908,7 @@
       <c r="C4" t="n">
         <v>1192.5</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>0.12</v>
       </c>
       <c r="E4" t="n">
@@ -1916,7 +1916,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1927,7 +1927,7 @@
       <c r="C5" t="n">
         <v>5578.5</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" t="n">
         <v>0.22</v>
       </c>
       <c r="E5" t="n">
@@ -1935,7 +1935,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1946,7 +1946,7 @@
       <c r="C6" t="n">
         <v>17651</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" t="n">
         <v>0.24</v>
       </c>
       <c r="E6" t="n">
@@ -1954,7 +1954,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1965,7 +1965,7 @@
       <c r="C7" t="n">
         <v>40199</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" t="n">
         <v>0.32</v>
       </c>
       <c r="E7" t="n">
@@ -1973,7 +1973,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -1984,7 +1984,7 @@
       <c r="C8" t="n">
         <v>57231</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" t="n">
         <v>0.35</v>
       </c>
       <c r="E8" t="n">
@@ -1992,7 +1992,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2003,7 +2003,7 @@
       <c r="C9" t="n">
         <v>188770</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" t="n">
         <v>0.37</v>
       </c>
       <c r="E9" t="n">
@@ -2011,7 +2011,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2022,7 +2022,7 @@
       <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" t="n">
         <v>0.1</v>
       </c>
       <c r="E10" t="n">
@@ -2030,7 +2030,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2041,7 +2041,7 @@
       <c r="C11" t="n">
         <v>2385</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" t="n">
         <v>0.12</v>
       </c>
       <c r="E11" t="n">
@@ -2049,7 +2049,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2060,7 +2060,7 @@
       <c r="C12" t="n">
         <v>11157</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" t="n">
         <v>0.22</v>
       </c>
       <c r="E12" t="n">
@@ -2068,7 +2068,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2079,7 +2079,7 @@
       <c r="C13" t="n">
         <v>35302</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" t="n">
         <v>0.24</v>
       </c>
       <c r="E13" t="n">
@@ -2087,7 +2087,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2098,7 +2098,7 @@
       <c r="C14" t="n">
         <v>80398</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" t="n">
         <v>0.32</v>
       </c>
       <c r="E14" t="n">
@@ -2106,7 +2106,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2117,7 +2117,7 @@
       <c r="C15" t="n">
         <v>114462</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" t="n">
         <v>0.35</v>
       </c>
       <c r="E15" t="n">
@@ -2125,7 +2125,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2136,7 +2136,7 @@
       <c r="C16" t="n">
         <v>202154.5</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" t="n">
         <v>0.37</v>
       </c>
       <c r="E16" t="n">
@@ -2144,7 +2144,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2155,7 +2155,7 @@
       <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" t="n">
         <v>0.1</v>
       </c>
       <c r="E17" t="n">
@@ -2163,7 +2163,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2174,7 +2174,7 @@
       <c r="C18" t="n">
         <v>1192.5</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" t="n">
         <v>0.12</v>
       </c>
       <c r="E18" t="n">
@@ -2182,7 +2182,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2193,7 +2193,7 @@
       <c r="C19" t="n">
         <v>5578.5</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" t="n">
         <v>0.22</v>
       </c>
       <c r="E19" t="n">
@@ -2201,7 +2201,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2212,7 +2212,7 @@
       <c r="C20" t="n">
         <v>17651</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" t="n">
         <v>0.24</v>
       </c>
       <c r="E20" t="n">
@@ -2220,7 +2220,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2231,7 +2231,7 @@
       <c r="C21" t="n">
         <v>40199</v>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" t="n">
         <v>0.32</v>
       </c>
       <c r="E21" t="n">
@@ -2239,7 +2239,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2250,7 +2250,7 @@
       <c r="C22" t="n">
         <v>57231</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" t="n">
         <v>0.35</v>
       </c>
       <c r="E22" t="n">
@@ -2258,7 +2258,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2269,7 +2269,7 @@
       <c r="C23" t="n">
         <v>101077.25</v>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="D23" t="n">
         <v>0.37</v>
       </c>
       <c r="E23" t="n">
@@ -2277,7 +2277,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2288,7 +2288,7 @@
       <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" t="n">
         <v>0.1</v>
       </c>
       <c r="E24" t="n">
@@ -2296,7 +2296,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2307,7 +2307,7 @@
       <c r="C25" t="n">
         <v>1700</v>
       </c>
-      <c r="D25" s="2" t="n">
+      <c r="D25" t="n">
         <v>0.12</v>
       </c>
       <c r="E25" t="n">
@@ -2315,7 +2315,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2326,7 +2326,7 @@
       <c r="C26" t="n">
         <v>7442</v>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" t="n">
         <v>0.22</v>
       </c>
       <c r="E26" t="n">
@@ -2334,7 +2334,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2345,7 +2345,7 @@
       <c r="C27" t="n">
         <v>15912</v>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D27" t="n">
         <v>0.24</v>
       </c>
       <c r="E27" t="n">
@@ -2353,7 +2353,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2364,7 +2364,7 @@
       <c r="C28" t="n">
         <v>38460</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D28" t="n">
         <v>0.32</v>
       </c>
       <c r="E28" t="n">
@@ -2372,7 +2372,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2383,7 +2383,7 @@
       <c r="C29" t="n">
         <v>55484</v>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D29" t="n">
         <v>0.35</v>
       </c>
       <c r="E29" t="n">
@@ -2391,7 +2391,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2402,27 +2402,23 @@
       <c r="C30" t="n">
         <v>187031.5</v>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D30" t="n">
         <v>0.37</v>
       </c>
       <c r="E30" t="n">
         <v>22500</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-    </row>
+    <row r="31"/>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Table B: Federal Capital Gains Brackets</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2437,10 +2433,9 @@
           <t>LTCG Rate</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2451,10 +2446,9 @@
       <c r="C34" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2465,10 +2459,9 @@
       <c r="C35" t="n">
         <v>0.15</v>
       </c>
-      <c r="D35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2479,10 +2472,9 @@
       <c r="C36" t="n">
         <v>0.2</v>
       </c>
-      <c r="D36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2493,10 +2485,9 @@
       <c r="C37" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2507,10 +2498,9 @@
       <c r="C38" t="n">
         <v>0.15</v>
       </c>
-      <c r="D38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2521,10 +2511,9 @@
       <c r="C39" t="n">
         <v>0.2</v>
       </c>
-      <c r="D39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2535,10 +2524,9 @@
       <c r="C40" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2549,10 +2537,9 @@
       <c r="C41" t="n">
         <v>0.15</v>
       </c>
-      <c r="D41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -2563,10 +2550,9 @@
       <c r="C42" t="n">
         <v>0.2</v>
       </c>
-      <c r="D42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2577,10 +2563,9 @@
       <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2591,10 +2576,9 @@
       <c r="C44" t="n">
         <v>0.15</v>
       </c>
-      <c r="D44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -2605,22 +2589,17 @@
       <c r="C45" t="n">
         <v>0.2</v>
       </c>
-      <c r="D45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-    </row>
+    </row>
+    <row r="46"/>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Table C: California FTB Brackets</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2635,7 +2614,7 @@
           <t>Base Tax</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Marginal Rate</t>
         </is>
@@ -2652,7 +2631,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2663,7 +2642,7 @@
       <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="2" t="n">
+      <c r="D49" t="n">
         <v>0.01</v>
       </c>
       <c r="E49" t="n">
@@ -2674,7 +2653,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2685,7 +2664,7 @@
       <c r="C50" t="n">
         <v>110.79</v>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="D50" t="n">
         <v>0.02</v>
       </c>
       <c r="E50" t="n">
@@ -2696,7 +2675,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2707,7 +2686,7 @@
       <c r="C51" t="n">
         <v>414.49</v>
       </c>
-      <c r="D51" s="2" t="n">
+      <c r="D51" t="n">
         <v>0.04</v>
       </c>
       <c r="E51" t="n">
@@ -2718,7 +2697,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2729,7 +2708,7 @@
       <c r="C52" t="n">
         <v>1022.01</v>
       </c>
-      <c r="D52" s="2" t="n">
+      <c r="D52" t="n">
         <v>0.06</v>
       </c>
       <c r="E52" t="n">
@@ -2740,7 +2719,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2751,7 +2730,7 @@
       <c r="C53" t="n">
         <v>1987.41</v>
       </c>
-      <c r="D53" s="2" t="n">
+      <c r="D53" t="n">
         <v>0.08</v>
       </c>
       <c r="E53" t="n">
@@ -2762,7 +2741,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2773,7 +2752,7 @@
       <c r="C54" t="n">
         <v>3201.97</v>
       </c>
-      <c r="D54" s="2" t="n">
+      <c r="D54" t="n">
         <v>0.093</v>
       </c>
       <c r="E54" t="n">
@@ -2784,7 +2763,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2795,7 +2774,7 @@
       <c r="C55" t="n">
         <v>31036.19</v>
       </c>
-      <c r="D55" s="2" t="n">
+      <c r="D55" t="n">
         <v>0.103</v>
       </c>
       <c r="E55" t="n">
@@ -2806,7 +2785,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2817,7 +2796,7 @@
       <c r="C56" t="n">
         <v>38688.19</v>
       </c>
-      <c r="D56" s="2" t="n">
+      <c r="D56" t="n">
         <v>0.113</v>
       </c>
       <c r="E56" t="n">
@@ -2828,7 +2807,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -2839,7 +2818,7 @@
       <c r="C57" t="n">
         <v>72269.75</v>
       </c>
-      <c r="D57" s="2" t="n">
+      <c r="D57" t="n">
         <v>0.123</v>
       </c>
       <c r="E57" t="n">
@@ -2850,7 +2829,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2861,7 +2840,7 @@
       <c r="C58" t="n">
         <v>0</v>
       </c>
-      <c r="D58" s="2" t="n">
+      <c r="D58" t="n">
         <v>0.01</v>
       </c>
       <c r="E58" t="n">
@@ -2872,7 +2851,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2883,7 +2862,7 @@
       <c r="C59" t="n">
         <v>221.58</v>
       </c>
-      <c r="D59" s="2" t="n">
+      <c r="D59" t="n">
         <v>0.02</v>
       </c>
       <c r="E59" t="n">
@@ -2894,7 +2873,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2905,7 +2884,7 @@
       <c r="C60" t="n">
         <v>828.98</v>
       </c>
-      <c r="D60" s="2" t="n">
+      <c r="D60" t="n">
         <v>0.04</v>
       </c>
       <c r="E60" t="n">
@@ -2916,7 +2895,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2927,7 +2906,7 @@
       <c r="C61" t="n">
         <v>2044.02</v>
       </c>
-      <c r="D61" s="2" t="n">
+      <c r="D61" t="n">
         <v>0.06</v>
       </c>
       <c r="E61" t="n">
@@ -2938,7 +2917,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2949,7 +2928,7 @@
       <c r="C62" t="n">
         <v>3974.82</v>
       </c>
-      <c r="D62" s="2" t="n">
+      <c r="D62" t="n">
         <v>0.08</v>
       </c>
       <c r="E62" t="n">
@@ -2960,7 +2939,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2971,7 +2950,7 @@
       <c r="C63" t="n">
         <v>6403.94</v>
       </c>
-      <c r="D63" s="2" t="n">
+      <c r="D63" t="n">
         <v>0.093</v>
       </c>
       <c r="E63" t="n">
@@ -2982,7 +2961,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -2993,7 +2972,7 @@
       <c r="C64" t="n">
         <v>61972.37</v>
       </c>
-      <c r="D64" s="2" t="n">
+      <c r="D64" t="n">
         <v>0.103</v>
       </c>
       <c r="E64" t="n">
@@ -3004,7 +2983,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -3015,7 +2994,7 @@
       <c r="C65" t="n">
         <v>77276.52</v>
       </c>
-      <c r="D65" s="2" t="n">
+      <c r="D65" t="n">
         <v>0.113</v>
       </c>
       <c r="E65" t="n">
@@ -3026,7 +3005,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -3037,7 +3016,7 @@
       <c r="C66" t="n">
         <v>144439.65</v>
       </c>
-      <c r="D66" s="2" t="n">
+      <c r="D66" t="n">
         <v>0.123</v>
       </c>
       <c r="E66" t="n">
@@ -3048,7 +3027,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3059,7 +3038,7 @@
       <c r="C67" t="n">
         <v>0</v>
       </c>
-      <c r="D67" s="2" t="n">
+      <c r="D67" t="n">
         <v>0.01</v>
       </c>
       <c r="E67" t="n">
@@ -3070,7 +3049,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3081,7 +3060,7 @@
       <c r="C68" t="n">
         <v>221.73</v>
       </c>
-      <c r="D68" s="2" t="n">
+      <c r="D68" t="n">
         <v>0.02</v>
       </c>
       <c r="E68" t="n">
@@ -3092,7 +3071,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3103,7 +3082,7 @@
       <c r="C69" t="n">
         <v>828.87</v>
       </c>
-      <c r="D69" s="2" t="n">
+      <c r="D69" t="n">
         <v>0.04</v>
       </c>
       <c r="E69" t="n">
@@ -3114,7 +3093,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3125,7 +3104,7 @@
       <c r="C70" t="n">
         <v>1436.31</v>
       </c>
-      <c r="D70" s="2" t="n">
+      <c r="D70" t="n">
         <v>0.06</v>
       </c>
       <c r="E70" t="n">
@@ -3136,7 +3115,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3147,7 +3126,7 @@
       <c r="C71" t="n">
         <v>2401.59</v>
       </c>
-      <c r="D71" s="2" t="n">
+      <c r="D71" t="n">
         <v>0.08</v>
       </c>
       <c r="E71" t="n">
@@ -3158,7 +3137,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3169,7 +3148,7 @@
       <c r="C72" t="n">
         <v>3616.47</v>
       </c>
-      <c r="D72" s="2" t="n">
+      <c r="D72" t="n">
         <v>0.093</v>
       </c>
       <c r="E72" t="n">
@@ -3180,7 +3159,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3191,7 +3170,7 @@
       <c r="C73" t="n">
         <v>41394.74</v>
       </c>
-      <c r="D73" s="2" t="n">
+      <c r="D73" t="n">
         <v>0.103</v>
       </c>
       <c r="E73" t="n">
@@ -3202,7 +3181,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3213,7 +3192,7 @@
       <c r="C74" t="n">
         <v>51802.17</v>
       </c>
-      <c r="D74" s="2" t="n">
+      <c r="D74" t="n">
         <v>0.113</v>
       </c>
       <c r="E74" t="n">
@@ -3224,7 +3203,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3235,7 +3214,7 @@
       <c r="C75" t="n">
         <v>97472.92999999999</v>
       </c>
-      <c r="D75" s="2" t="n">
+      <c r="D75" t="n">
         <v>0.123</v>
       </c>
       <c r="E75" t="n">
@@ -3245,20 +3224,16 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="2" t="n"/>
-      <c r="D76" s="2" t="n"/>
-    </row>
+    <row r="76"/>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>Table D: Surtaxes &amp; Phaseouts</t>
         </is>
       </c>
-      <c r="D77" s="2" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -3273,14 +3248,14 @@
           <t>Addl Medicare</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>CTC Phaseout Start</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -3291,12 +3266,12 @@
       <c r="C79" t="n">
         <v>200000</v>
       </c>
-      <c r="D79" s="2" t="n">
+      <c r="D79" t="n">
         <v>200000</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>MFJ</t>
         </is>
@@ -3307,12 +3282,12 @@
       <c r="C80" t="n">
         <v>250000</v>
       </c>
-      <c r="D80" s="2" t="n">
+      <c r="D80" t="n">
         <v>400000</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>MFS</t>
         </is>
@@ -3323,12 +3298,12 @@
       <c r="C81" t="n">
         <v>125000</v>
       </c>
-      <c r="D81" s="2" t="n">
+      <c r="D81" t="n">
         <v>200000</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>HoH</t>
         </is>
@@ -3339,7 +3314,7 @@
       <c r="C82" t="n">
         <v>200000</v>
       </c>
-      <c r="D82" s="2" t="n">
+      <c r="D82" t="n">
         <v>200000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Instructions tab off-by-one: Highlighted row 8 (Important Notes) instead of row 9
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -609,14 +609,14 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Important Notes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1. Investment Income: All dividends and interest are combined and taxed as Ordinary Income for a safe, conservative projection.</t>
         </is>

</xml_diff>

<commit_message>
Restored Filing Status dropdown selector in cell B2
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -1708,6 +1708,11 @@
       <c r="I64" s="2" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
+      <formula1>"Single,MFJ,MFS,HoH"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed HSA false positive: System now correctly identifies users without an HSA and displays 'No HSA Detected'
</commit_message>
<xml_diff>
--- a/Tax_Orchestrator_Template.xlsx
+++ b/Tax_Orchestrator_Template.xlsx
@@ -265,7 +265,7 @@
     </comment>
     <comment ref="I28" authorId="0" shapeId="0">
       <text>
-        <t>Confirms that HSA contributions are successfully added back to California income (as they are not deductible at the state level).</t>
+        <t>HSA Verification: Checks that HSA contributions are added back to California income. If you do not have an HSA, this will simply confirm 'No HSA Detected'.</t>
       </text>
     </comment>
   </commentList>
@@ -665,7 +665,7 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1264,11 +1264,11 @@
       <c r="D28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>HSA Audit (CA):</t>
+          <t>HSA Verification (CA):</t>
         </is>
       </c>
       <c r="J28">
-        <f>IF(B20=B19, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)")</f>
+        <f>IF(SUM('Wage Snapshots'!D:D)=0, "✅ No HSA Detected", IF(B20=B19, "🔴 ERR: HSA NOT ADDED TO CA", "✅ HSA Corrected (CA)"))</f>
         <v/>
       </c>
     </row>

</xml_diff>